<commit_message>
Use real-format sanitized templates for the demo pair
Replace the hand-built demo PO with one derived from a real Oracle XML
Publisher export, trimmed to two orders and fully sanitized in place so
it keeps the exact original HTML/CSS/layout users will see in practice.
All real data (company, addresses, contacts, emails, phones, part
numbers, customers, commission rates, prices, PO numbers) is replaced
with demo/example.com values; verified by full-fragment review (0 real
tokens) and an end-to-end run (5 lines matched, 2 totals recomputed).
Ship list updated to the matching demo keys.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/出貨清單_範本.xlsx
+++ b/出貨清單_範本.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -453,7 +453,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1200</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3">
@@ -467,29 +467,65 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ITEM-DEMO-B</t>
+          <t>ITEM-DEMO-A</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>500</v>
+        <v>88</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>PO-DEMO-001</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ITEM-DEMO-A</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>PO-DEMO-001</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ITEM-DEMO-A</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t>PO-DEMO-002</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B6" t="n">
         <v>1</v>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>ITEM-DEMO-D</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>900</v>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ITEM-DEMO-B</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>